<commit_message>
Added a new library preparation kit: 10x Genomics; Chromium Next GEM Single Cell Fixed RNA Sample Preparation Kit, 16 rxns; PN 1000414
Closes #153
</commit_message>
<xml_diff>
--- a/rnaseq/latest/rnaseq.xlsx
+++ b/rnaseq/latest/rnaseq.xlsx
@@ -47,6 +47,11 @@
   <commentList>
     <comment ref="A1" authorId="1">
       <text>
+        <t>A styled paragraph describing the assay</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="1">
+      <text>
         <t>(Required) The unique identifier from HuBMAP or SenNet for the sample (such as a
 block, section, or suspension) used to perform the assay. For instance, in an
 RNAseq assay, the parent sample would be the suspension, while in imaging
@@ -55,7 +60,7 @@
 Example: HBM386.ZGKG.235, HBM672.MKPK.442</t>
       </text>
     </comment>
-    <comment ref="B1" authorId="1">
+    <comment ref="C1" authorId="1">
       <text>
         <t>A locally assigned identifier provided by the data provider for the dataset. It
 is used to reference an external metadata record that may be maintained
@@ -63,7 +68,7 @@
 Example: Visium_9OLC_A4_S1</t>
       </text>
     </comment>
-    <comment ref="C1" authorId="1">
+    <comment ref="D1" authorId="1">
       <text>
         <t>(Required) The DOI for the protocols.io page that details the assay or the
 procedures used for sample procurement and preparation. For example, in the case
@@ -73,24 +78,24 @@
 Example: https://dx.doi.org/10.17504/protocols.io.eq2lyno9qvx9/v1</t>
       </text>
     </comment>
-    <comment ref="D1" authorId="1">
+    <comment ref="E1" authorId="1">
       <text>
         <t>(Required) The specific type of dataset being produced. Example: RNAseq</t>
       </text>
     </comment>
-    <comment ref="E1" authorId="1">
+    <comment ref="F1" authorId="1">
       <text>
         <t>(Required) The analyte class which is the target molecule that the assay is
 measuring. Example: DNA</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="1">
+    <comment ref="G1" authorId="1">
       <text>
         <t>(Required) Indicates whether a specific molecule or set of molecules is targeted
 for detection or measurement by the assay. Example: Yes</t>
       </text>
     </comment>
-    <comment ref="G1" authorId="1">
+    <comment ref="H1" authorId="1">
       <text>
         <t>(Required) The company that manufactures or supplies the acquisition instrument.
 An acquisition instrument is a device equipped with signal detection hardware
@@ -100,7 +105,7 @@
 "In-House". Example: Illumina</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="1">
+    <comment ref="I1" authorId="1">
       <text>
         <t>(Required) The specific model of the acquisition instrument, as manufacturers
 often offer various versions with differing features or sensitivities. These
@@ -109,7 +114,7 @@
 the model is unknown, enter "Unknown". Example: HiSeq 4000</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="1">
+    <comment ref="J1" authorId="1">
       <text>
         <t>(Required) The length of time the sample was stored prior to processing it. For
 assays performed on tissue sections, this refers to how long the tissue section
@@ -118,32 +123,32 @@
 suspension was stored before library construction started. Example: 12</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="1">
+    <comment ref="K1" authorId="1">
       <text>
         <t>(Required) The unit of measurement used to specify the source storage duration
 value. Example: hour</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="1">
+    <comment ref="L1" authorId="1">
       <text>
         <t>The length of time since the acquisition instrument was last serviced or
 calibrated. This provides a metric for assessing drift in data capture. Example:
 10</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="1">
+    <comment ref="M1" authorId="1">
       <text>
         <t>The unit of measurement used to specify the time since acquisition instrument
 calibration value. Example: month</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="1">
+    <comment ref="N1" authorId="1">
       <text>
         <t>(Required) The name of the file containing the ORCID IDs for all contributors to
 this dataset. Example: ./contributors.csv</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="1">
+    <comment ref="O1" authorId="1">
       <text>
         <t>(Required) The top-level directory containing the raw and/or processed data. For
 a single dataset upload, this might be represented as ".", whereas for a data
@@ -155,7 +160,7 @@
 an internal metadata field used solely for data ingestion. Example: ./TEST001-RK</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="1">
+    <comment ref="P1" authorId="1">
       <text>
         <t>(Required) The position within a sequencing read where a barcode sequence
 begins. In sequencing libraries, barcodes—short DNA sequences used to tag
@@ -168,7 +173,7 @@
 Example: 0,38,76</t>
       </text>
     </comment>
-    <comment ref="P1" authorId="1">
+    <comment ref="Q1" authorId="1">
       <text>
         <t>(Required) The sequencing read file contains the cell or capture spot barcode
 sequences. This information is essential when constructing sequencing libraries
@@ -177,13 +182,13 @@
 should be marked as "Not applicable". Example: Read 1 (R1)</t>
       </text>
     </comment>
-    <comment ref="Q1" authorId="1">
+    <comment ref="R1" authorId="1">
       <text>
         <t>(Required) The length of each cell or capture spot barcode in base pairs (bp).
 If the source material is not barcoded, enter "Not applicable". Example: 16</t>
       </text>
     </comment>
-    <comment ref="R1" authorId="1">
+    <comment ref="S1" authorId="1">
       <text>
         <t>(Required) The position within a sequencing read where the Unique Molecular
 Identifier (UMI) sequence begins. UMIs are short, random nucleotide sequences
@@ -191,34 +196,34 @@
 original molecule. If no UMI is used, enter "Not applicable". Example: 16</t>
       </text>
     </comment>
-    <comment ref="S1" authorId="1">
+    <comment ref="T1" authorId="1">
       <text>
         <t>(Required) Specifies which sequencing read file contains the Unique Molecular
 Identifier (UMI) barcode. If no UMI is used, enter "Not applicable". Example:
 Read 1 (R1)</t>
       </text>
     </comment>
-    <comment ref="T1" authorId="1">
+    <comment ref="U1" authorId="1">
       <text>
         <t>(Required) The length of the Unique Molecular Identifier (UMI) in base pairs
 (bp). If no UMI is used, enter "Not applicable". Example: 8</t>
       </text>
     </comment>
-    <comment ref="U1" authorId="1">
+    <comment ref="V1" authorId="1">
       <text>
         <t>(Required) The entity from which the analyte is captured. For example, in bulk
 sequencing, the source entity would be "tissue" while in single-cell sequencing,
 it would be "single cell". Example: single cell</t>
       </text>
     </comment>
-    <comment ref="V1" authorId="1">
+    <comment ref="W1" authorId="1">
       <text>
         <t>The number of cells or nuclei that were input into the assay. This information
 is typically not available for assays performed on bulk tissue preparations, and
 therefore this field may be left blank. Example: 1000</t>
       </text>
     </comment>
-    <comment ref="W1" authorId="1">
+    <comment ref="X1" authorId="1">
       <text>
         <t>The amount of RNA or DNA input into the assay, typically measured using
 instruments such as a Qubit, BioAnalyzer, or TapeStation. In most single-cell or
@@ -226,13 +231,13 @@
 field may be left blank. Example: 500</t>
       </text>
     </comment>
-    <comment ref="X1" authorId="1">
+    <comment ref="Y1" authorId="1">
       <text>
         <t>The unit of measurement used to specify the amount of input analyte value. If no
 input amount, this field may be left blank. Example: ng</t>
       </text>
     </comment>
-    <comment ref="Y1" authorId="1">
+    <comment ref="Z1" authorId="1">
       <text>
         <t>(Required) The 5' and/or 3' adapter sequences used during library preparation to
 make the library compatible with the sequencing protocol and instrumentation.
@@ -241,57 +246,57 @@
 CTGTCTCTTATACACATCT</t>
       </text>
     </comment>
-    <comment ref="Z1" authorId="1">
+    <comment ref="AA1" authorId="1">
       <text>
         <t>(Required) The average size of sequencing library fragments, measured in base
 pairs (bp), as estimated by gel electrophoresis, BioAnalyzer, or TapeStation.
 Example: 200</t>
       </text>
     </comment>
-    <comment ref="AA1" authorId="1">
+    <comment ref="AB1" authorId="1">
       <text>
         <t>(Required) The amount of cDNA, after amplification, that was used for library
 construction. Example: 60</t>
       </text>
     </comment>
-    <comment ref="AB1" authorId="1">
+    <comment ref="AC1" authorId="1">
       <text>
         <t>(Required) The unit of measurement used to specify the library input amount
 value. Example: ng</t>
       </text>
     </comment>
-    <comment ref="AC1" authorId="1">
+    <comment ref="AD1" authorId="1">
       <text>
         <t>The total amount of library following the clean-up step after the final PCR
 amplification. To calculate, multiply the Qubit-measured concentration (ng/µl)
 by the elution volume (µl) obtained after the final clean-up. Example: 125</t>
       </text>
     </comment>
-    <comment ref="AD1" authorId="1">
+    <comment ref="AE1" authorId="1">
       <text>
         <t>The unit of measurement used to specify the library output amount value.
 Example: ng</t>
       </text>
     </comment>
-    <comment ref="AE1" authorId="1">
+    <comment ref="AF1" authorId="1">
       <text>
         <t>(Required) The concentration of the pooled library submitted for sequencing.
 Example: 2.5</t>
       </text>
     </comment>
-    <comment ref="AF1" authorId="1">
+    <comment ref="AG1" authorId="1">
       <text>
         <t>(Required) Unit of library concentration value.</t>
       </text>
     </comment>
-    <comment ref="AG1" authorId="1">
+    <comment ref="AH1" authorId="1">
       <text>
         <t>(Required) Indicates whether the sequencing library was prepared for single-end
 or paired-end sequencing. This information determines how reads are generated
 and aligned during data processing. Example: single-end</t>
       </text>
     </comment>
-    <comment ref="AH1" authorId="1">
+    <comment ref="AI1" authorId="1">
       <text>
         <t>(Required) The number of amplification cycles applied to cDNA prior to library
 construction. This is typically the number of PCR cycles used. For protocols
@@ -299,7 +304,7 @@
 amplification rounds performed. Example: 3</t>
       </text>
     </comment>
-    <comment ref="AI1" authorId="1">
+    <comment ref="AJ1" authorId="1">
       <text>
         <t>(Required) The number of PCR cycles used specifically to add sequencing adapters
 and amplify the library during the indexing step. This count does not include
@@ -307,7 +312,7 @@
 "Number of iterations of cDNA amplification" field. Example: 8</t>
       </text>
     </comment>
-    <comment ref="AJ1" authorId="1">
+    <comment ref="AK1" authorId="1">
       <text>
         <t>(Required) The reagent kit used to construct the sequencing library, including
 both the kit name and, if available, version and product number. If the library
@@ -315,7 +320,7 @@
 Chromium Next GEM Single Cell 5' Kit v2, 16 rxns; PN 1000263</t>
       </text>
     </comment>
-    <comment ref="AK1" authorId="1">
+    <comment ref="AL1" authorId="1">
       <text>
         <t>(Required) The reagent kit used to add index sequences to samples. Indexes
 enable multiplexing, allowing multiple libraries to be pooled and sequenced
@@ -327,27 +332,27 @@
 1000251</t>
       </text>
     </comment>
-    <comment ref="AL1" authorId="1">
+    <comment ref="AM1" authorId="1">
       <text>
         <t>(Required) The specific sequencing barcode index set used, chosen from the
 sample indexing kit. For example, in the case of 10x, this might be "SI-GA-A1",
 whereas for Nextera, it could be "N505 - CTCCTTAC". Example: SI-GA-A1</t>
       </text>
     </comment>
-    <comment ref="AM1" authorId="1">
+    <comment ref="AN1" authorId="1">
       <text>
         <t>(Required) Indicates whether the sequencing reaction was run in replicate. If
 "Yes," the corresponding FASTQ files in the dataset should be merged for
 analysis. Example: Yes</t>
       </text>
     </comment>
-    <comment ref="AN1" authorId="1">
+    <comment ref="AO1" authorId="1">
       <text>
         <t>The number of cells, nuclei, or capture spots expected to be captured by the
 assay. Example: 14336</t>
       </text>
     </comment>
-    <comment ref="AO1" authorId="1">
+    <comment ref="AP1" authorId="1">
       <text>
         <t>(Required) The reagent kit used to perform the sequencing run, including the
 platform, kit name, version, and product number when available. If the reagent
@@ -355,14 +360,14 @@
 NextSeq 500/550 Hi Output Kit 150 Cycles; v2.5; PN 20024907</t>
       </text>
     </comment>
-    <comment ref="AP1" authorId="1">
+    <comment ref="AQ1" authorId="1">
       <text>
         <t>(Required) The number of sequencing cycles for each read and index in the
 sequencing run, typically reported as a comma-separated list in the order: Read
 1, i7 index, i5 index, and Read 2. Example: 50,8,16,50</t>
       </text>
     </comment>
-    <comment ref="AQ1" authorId="1">
+    <comment ref="AR1" authorId="1">
       <text>
         <t>A lab-assigned identifier for the sequencing run, such as a chip ID, that
 enables users to determine which samples were processed together. To avoid ID
@@ -370,7 +375,7 @@
 of the sequencing center. Example: Broad_Chip1234</t>
       </text>
     </comment>
-    <comment ref="AR1" authorId="1">
+    <comment ref="AS1" authorId="1">
       <text>
         <t>A lab-assigned identifier used to indicate which cells or nuclei were captured
 together in the same run. For example, in a 10X Genomics Chromium Controller
@@ -380,7 +385,7 @@
 the ID with the name of the sequencing center. Example: Broad_Batch1234</t>
       </text>
     </comment>
-    <comment ref="AS1" authorId="1">
+    <comment ref="AT1" authorId="1">
       <text>
         <t>The company that manufactures the instrument used to prepare the sample (e.g.,
 for staining or other processing steps) prior to the assay. If the instrument
@@ -388,7 +393,7 @@
 preparation occurred, enter "Not applicable". Example: 10X Genomics</t>
       </text>
     </comment>
-    <comment ref="AT1" authorId="1">
+    <comment ref="AU1" authorId="1">
       <text>
         <t>The specific model of the instrument used for sample preparation, such as
 staining. Manufacturers may offer multiple models with varying features or
@@ -397,7 +402,7 @@
 applicable". Example: Chromium X</t>
       </text>
     </comment>
-    <comment ref="AU1" authorId="1">
+    <comment ref="AV1" authorId="1">
       <text>
         <t>The reagent kit used in conjunction with the preparation instrument for sample
 processing (e.g., staining or labeling). If the reagent kit was prepared using a
@@ -405,7 +410,7 @@
 Single Cell Kit, 48 rxns; PN 1000120</t>
       </text>
     </comment>
-    <comment ref="AV1" authorId="1">
+    <comment ref="AW1" authorId="1">
       <text>
         <t>(Required) The unique string identifier for the metadata specification version,
 which is easily interpretable by computers for purposes of data validation and
@@ -417,7 +422,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="678">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="715">
+  <si>
+    <t>assay_description</t>
+  </si>
   <si>
     <t>parent_sample_id</t>
   </si>
@@ -521,6 +529,12 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000168</t>
   </si>
   <si>
+    <t>iCLAP</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000479</t>
+  </si>
+  <si>
     <t>seqFISH</t>
   </si>
   <si>
@@ -587,6 +601,12 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000207</t>
   </si>
   <si>
+    <t>MACSima</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000480</t>
+  </si>
+  <si>
     <t>CyTOF</t>
   </si>
   <si>
@@ -719,6 +739,12 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000301</t>
   </si>
   <si>
+    <t>Raman Imaging</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000475</t>
+  </si>
+  <si>
     <t>RNAseq (with probes)</t>
   </si>
   <si>
@@ -731,6 +757,12 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000405</t>
   </si>
   <si>
+    <t>STARmap</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000476</t>
+  </si>
+  <si>
     <t>MPLEx</t>
   </si>
   <si>
@@ -758,6 +790,12 @@
     <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C13201</t>
   </si>
   <si>
+    <t>Lipid + metabolite + protein</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000478</t>
+  </si>
+  <si>
     <t>RNA + protein</t>
   </si>
   <si>
@@ -944,6 +982,12 @@
     <t>https://identifiers.org/RRID:SCR_023605</t>
   </si>
   <si>
+    <t>Waters</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024589</t>
+  </si>
+  <si>
     <t>In-House</t>
   </si>
   <si>
@@ -998,12 +1042,24 @@
     <t>https://identifiers.org/RRID:SCR_023604</t>
   </si>
   <si>
+    <t>Miltenyi Biotec</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_008984</t>
+  </si>
+  <si>
     <t>Leica Biosystems</t>
   </si>
   <si>
     <t>https://identifiers.org/RRID:SCR_023603</t>
   </si>
   <si>
+    <t>Revvity</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027779</t>
+  </si>
+  <si>
     <t>Cytek Biosciences</t>
   </si>
   <si>
@@ -1085,6 +1141,12 @@
     <t>https://identifiers.org/RRID:SCR_024569</t>
   </si>
   <si>
+    <t>LSM 710 Confocal Microscope</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_018063</t>
+  </si>
+  <si>
     <t>NanoZoomer 2.0-HT</t>
   </si>
   <si>
@@ -1133,6 +1195,18 @@
     <t>https://identifiers.org/RRID:SCR_026452</t>
   </si>
   <si>
+    <t>DMi8</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026672</t>
+  </si>
+  <si>
+    <t>Opera Phenix Plus HCS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027780</t>
+  </si>
+  <si>
     <t>timsTOF Pro 2</t>
   </si>
   <si>
@@ -1175,6 +1249,12 @@
     <t>https://identifiers.org/RRID:SCR_027101</t>
   </si>
   <si>
+    <t>Orbitrap Fusion Tribrid</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020559</t>
+  </si>
+  <si>
     <t>Custom: Multiphoton</t>
   </si>
   <si>
@@ -1301,6 +1381,18 @@
     <t>https://identifiers.org/RRID:SCR_027072</t>
   </si>
   <si>
+    <t>Opera Phenix HCS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027817</t>
+  </si>
+  <si>
+    <t>Zeiss LightSheet Z.1</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020919</t>
+  </si>
+  <si>
     <t>IN Cell Analyzer 2200</t>
   </si>
   <si>
@@ -1373,6 +1465,12 @@
     <t>https://identifiers.org/RRID:SCR_023692</t>
   </si>
   <si>
+    <t>NanoZoomer 2.0-RS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_028001</t>
+  </si>
+  <si>
     <t>Axio Observer 3</t>
   </si>
   <si>
@@ -1442,6 +1540,18 @@
     <t>https://identifiers.org/RRID:SCR_023613</t>
   </si>
   <si>
+    <t>SYNAPT G2-Si</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027782</t>
+  </si>
+  <si>
+    <t>MACSima System</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027923</t>
+  </si>
+  <si>
     <t>Biomark HD</t>
   </si>
   <si>
@@ -1757,6 +1867,12 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000366</t>
   </si>
   <si>
+    <t>10x Genomics; Chromium Next GEM Single Cell Fixed RNA Sample Preparation Kit, 16 rxns; PN 1000414</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000484</t>
+  </si>
+  <si>
     <t>10X Genomics; Visium Spatial Gene Expression Slide and Reagent Kit, 4 slides, 16 reactions; PN 1000184</t>
   </si>
   <si>
@@ -2444,7 +2560,7 @@
     <t>pav:createdOn</t>
   </si>
   <si>
-    <t>2025-11-20T09:40:56-08:00</t>
+    <t>2026-03-13T14:28:47-07:00</t>
   </si>
   <si>
     <t>pav:derivedFrom</t>
@@ -2503,11 +2619,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyAlignment="true" applyFill="true">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2566,57 +2683,58 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AV2"/>
+  <dimension ref="A1:AW2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" style="2" width="14.39453125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" style="3" width="5.46875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" style="4" width="20.234375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" style="5" width="10.59765625" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" style="6" width="10.9296875" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" style="7" width="9.40234375" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" style="8" width="24.5546875" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" style="9" width="24.0390625" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" style="10" width="24.63671875" customWidth="true" bestFit="true"/>
-    <col min="10" max="10" style="11" width="23.63671875" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" style="12" width="41.1015625" customWidth="true" bestFit="true"/>
-    <col min="12" max="12" style="13" width="40.1015625" customWidth="true" bestFit="true"/>
-    <col min="13" max="13" style="14" width="14.5859375" customWidth="true" bestFit="true"/>
-    <col min="14" max="14" style="15" width="8.46484375" customWidth="true" bestFit="true"/>
-    <col min="15" max="15" style="16" width="12.27734375" customWidth="true" bestFit="true"/>
-    <col min="16" max="16" style="17" width="11.26171875" customWidth="true" bestFit="true"/>
-    <col min="17" max="17" style="18" width="10.9140625" customWidth="true" bestFit="true"/>
-    <col min="18" max="18" style="19" width="9.01953125" customWidth="true" bestFit="true"/>
-    <col min="19" max="19" style="20" width="8.00390625" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" style="21" width="7.65625" customWidth="true" bestFit="true"/>
-    <col min="21" max="21" style="22" width="15.00390625" customWidth="true" bestFit="true"/>
-    <col min="22" max="22" style="23" width="25.9765625" customWidth="true" bestFit="true"/>
-    <col min="23" max="23" style="24" width="24.99609375" customWidth="true" bestFit="true"/>
-    <col min="24" max="24" style="25" width="23.99609375" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" style="26" width="20.4609375" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" style="27" width="24.20703125" customWidth="true" bestFit="true"/>
-    <col min="27" max="27" style="28" width="22.0703125" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" style="29" width="21.0703125" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" style="30" width="23.17578125" customWidth="true" bestFit="true"/>
-    <col min="30" max="30" style="31" width="22.17578125" customWidth="true" bestFit="true"/>
-    <col min="31" max="31" style="32" width="21.9453125" customWidth="true" bestFit="true"/>
-    <col min="32" max="32" style="33" width="20.9453125" customWidth="true" bestFit="true"/>
-    <col min="33" max="33" style="34" width="11.296875" customWidth="true" bestFit="true"/>
-    <col min="34" max="34" style="35" width="34.82421875" customWidth="true" bestFit="true"/>
-    <col min="35" max="35" style="36" width="28.32421875" customWidth="true" bestFit="true"/>
-    <col min="36" max="36" style="37" width="18.2734375" customWidth="true" bestFit="true"/>
-    <col min="37" max="37" style="38" width="16.65234375" customWidth="true" bestFit="true"/>
-    <col min="38" max="38" style="39" width="16.9609375" customWidth="true" bestFit="true"/>
-    <col min="39" max="39" style="40" width="17.18359375" customWidth="true" bestFit="true"/>
-    <col min="40" max="40" style="41" width="24.72265625" customWidth="true" bestFit="true"/>
-    <col min="41" max="41" style="42" width="19.05859375" customWidth="true" bestFit="true"/>
-    <col min="42" max="42" style="43" width="19.78125" customWidth="true" bestFit="true"/>
-    <col min="43" max="43" style="44" width="16.94921875" customWidth="true" bestFit="true"/>
-    <col min="44" max="44" style="45" width="13.96484375" customWidth="true" bestFit="true"/>
-    <col min="45" max="45" style="46" width="25.0859375" customWidth="true" bestFit="true"/>
-    <col min="46" max="46" style="47" width="24.57421875" customWidth="true" bestFit="true"/>
-    <col min="47" max="47" style="48" width="21.765625" customWidth="true" bestFit="true"/>
-    <col min="48" max="48" style="49" width="16.91796875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" style="2" width="14.46875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="2" max="2" style="3" width="14.39453125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" style="4" width="5.46875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" style="5" width="20.234375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" style="6" width="10.59765625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" style="7" width="10.9296875" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" style="8" width="9.40234375" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" style="9" width="24.5546875" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" style="10" width="24.0390625" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" style="11" width="24.63671875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" style="12" width="23.63671875" customWidth="true" bestFit="true"/>
+    <col min="12" max="12" style="13" width="41.1015625" customWidth="true" bestFit="true"/>
+    <col min="13" max="13" style="14" width="40.1015625" customWidth="true" bestFit="true"/>
+    <col min="14" max="14" style="15" width="14.5859375" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" style="16" width="8.46484375" customWidth="true" bestFit="true"/>
+    <col min="16" max="16" style="17" width="12.27734375" customWidth="true" bestFit="true"/>
+    <col min="17" max="17" style="18" width="11.26171875" customWidth="true" bestFit="true"/>
+    <col min="18" max="18" style="19" width="10.9140625" customWidth="true" bestFit="true"/>
+    <col min="19" max="19" style="20" width="9.01953125" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" style="21" width="8.00390625" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" style="22" width="7.65625" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" style="23" width="15.00390625" customWidth="true" bestFit="true"/>
+    <col min="23" max="23" style="24" width="25.9765625" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" style="25" width="24.99609375" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" style="26" width="23.99609375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" style="27" width="20.4609375" customWidth="true" bestFit="true"/>
+    <col min="27" max="27" style="28" width="24.20703125" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" style="29" width="22.0703125" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" style="30" width="21.0703125" customWidth="true" bestFit="true"/>
+    <col min="30" max="30" style="31" width="23.17578125" customWidth="true" bestFit="true"/>
+    <col min="31" max="31" style="32" width="22.17578125" customWidth="true" bestFit="true"/>
+    <col min="32" max="32" style="33" width="21.9453125" customWidth="true" bestFit="true"/>
+    <col min="33" max="33" style="34" width="20.9453125" customWidth="true" bestFit="true"/>
+    <col min="34" max="34" style="35" width="11.296875" customWidth="true" bestFit="true"/>
+    <col min="35" max="35" style="36" width="34.82421875" customWidth="true" bestFit="true"/>
+    <col min="36" max="36" style="37" width="28.32421875" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" style="38" width="18.2734375" customWidth="true" bestFit="true"/>
+    <col min="38" max="38" style="39" width="16.65234375" customWidth="true" bestFit="true"/>
+    <col min="39" max="39" style="40" width="16.9609375" customWidth="true" bestFit="true"/>
+    <col min="40" max="40" style="41" width="17.18359375" customWidth="true" bestFit="true"/>
+    <col min="41" max="41" style="42" width="24.72265625" customWidth="true" bestFit="true"/>
+    <col min="42" max="42" style="43" width="19.05859375" customWidth="true" bestFit="true"/>
+    <col min="43" max="43" style="44" width="19.78125" customWidth="true" bestFit="true"/>
+    <col min="44" max="44" style="45" width="16.94921875" customWidth="true" bestFit="true"/>
+    <col min="45" max="45" style="46" width="13.96484375" customWidth="true" bestFit="true"/>
+    <col min="46" max="46" style="47" width="25.0859375" customWidth="true" bestFit="true"/>
+    <col min="47" max="47" style="48" width="24.57421875" customWidth="true" bestFit="true"/>
+    <col min="48" max="48" style="49" width="21.765625" customWidth="true" bestFit="true"/>
+    <col min="49" max="49" style="50" width="16.91796875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2633,268 +2751,271 @@
         <v>3</v>
       </c>
       <c r="E1" t="s" s="1">
-        <v>106</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s" s="1">
-        <v>141</v>
+        <v>115</v>
       </c>
       <c r="G1" t="s" s="1">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="H1" t="s" s="1">
-        <v>205</v>
+        <v>155</v>
       </c>
       <c r="I1" t="s" s="1">
-        <v>357</v>
+        <v>222</v>
       </c>
       <c r="J1" t="s" s="1">
-        <v>358</v>
+        <v>392</v>
       </c>
       <c r="K1" t="s" s="1">
-        <v>369</v>
+        <v>393</v>
       </c>
       <c r="L1" t="s" s="1">
-        <v>370</v>
+        <v>404</v>
       </c>
       <c r="M1" t="s" s="1">
-        <v>371</v>
+        <v>405</v>
       </c>
       <c r="N1" t="s" s="1">
-        <v>372</v>
+        <v>406</v>
       </c>
       <c r="O1" t="s" s="1">
-        <v>373</v>
+        <v>407</v>
       </c>
       <c r="P1" t="s" s="1">
-        <v>382</v>
+        <v>408</v>
       </c>
       <c r="Q1" t="s" s="1">
-        <v>387</v>
+        <v>417</v>
       </c>
       <c r="R1" t="s" s="1">
-        <v>393</v>
+        <v>422</v>
       </c>
       <c r="S1" t="s" s="1">
-        <v>395</v>
+        <v>428</v>
       </c>
       <c r="T1" t="s" s="1">
-        <v>396</v>
+        <v>430</v>
       </c>
       <c r="U1" t="s" s="1">
-        <v>400</v>
+        <v>431</v>
       </c>
       <c r="V1" t="s" s="1">
-        <v>411</v>
+        <v>435</v>
       </c>
       <c r="W1" t="s" s="1">
-        <v>412</v>
+        <v>446</v>
       </c>
       <c r="X1" t="s" s="1">
-        <v>413</v>
+        <v>447</v>
       </c>
       <c r="Y1" t="s" s="1">
-        <v>418</v>
+        <v>448</v>
       </c>
       <c r="Z1" t="s" s="1">
-        <v>419</v>
+        <v>453</v>
       </c>
       <c r="AA1" t="s" s="1">
-        <v>420</v>
+        <v>454</v>
       </c>
       <c r="AB1" t="s" s="1">
-        <v>421</v>
+        <v>455</v>
       </c>
       <c r="AC1" t="s" s="1">
-        <v>424</v>
+        <v>456</v>
       </c>
       <c r="AD1" t="s" s="1">
-        <v>425</v>
+        <v>459</v>
       </c>
       <c r="AE1" t="s" s="1">
-        <v>426</v>
+        <v>460</v>
       </c>
       <c r="AF1" t="s" s="1">
-        <v>427</v>
+        <v>461</v>
       </c>
       <c r="AG1" t="s" s="1">
-        <v>434</v>
+        <v>462</v>
       </c>
       <c r="AH1" t="s" s="1">
-        <v>439</v>
+        <v>469</v>
       </c>
       <c r="AI1" t="s" s="1">
-        <v>440</v>
+        <v>474</v>
       </c>
       <c r="AJ1" t="s" s="1">
-        <v>441</v>
+        <v>475</v>
       </c>
       <c r="AK1" t="s" s="1">
-        <v>516</v>
+        <v>476</v>
       </c>
       <c r="AL1" t="s" s="1">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="AM1" t="s" s="1">
-        <v>552</v>
+        <v>588</v>
       </c>
       <c r="AN1" t="s" s="1">
-        <v>553</v>
+        <v>589</v>
       </c>
       <c r="AO1" t="s" s="1">
-        <v>554</v>
+        <v>590</v>
       </c>
       <c r="AP1" t="s" s="1">
-        <v>611</v>
+        <v>591</v>
       </c>
       <c r="AQ1" t="s" s="1">
-        <v>612</v>
+        <v>648</v>
       </c>
       <c r="AR1" t="s" s="1">
-        <v>613</v>
+        <v>649</v>
       </c>
       <c r="AS1" t="s" s="1">
-        <v>614</v>
+        <v>650</v>
       </c>
       <c r="AT1" t="s" s="1">
-        <v>621</v>
+        <v>651</v>
       </c>
       <c r="AU1" t="s" s="1">
-        <v>648</v>
+        <v>658</v>
       </c>
       <c r="AV1" t="s" s="1">
-        <v>669</v>
+        <v>685</v>
+      </c>
+      <c r="AW1" t="s" s="1">
+        <v>706</v>
       </c>
     </row>
     <row r="2">
-      <c r="D2" t="s" s="5">
-        <v>92</v>
-      </c>
-      <c r="AV2" t="s" s="49">
-        <v>670</v>
+      <c r="E2" t="s" s="6">
+        <v>97</v>
+      </c>
+      <c r="AW2" t="s" s="50">
+        <v>707</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="37">
-    <dataValidation type="list" sqref="D2:D1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'dataset_type'!$A$1:$A$51</formula1>
-    </dataValidation>
     <dataValidation type="list" sqref="E2:E1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'analyte_class'!$A$1:$A$17</formula1>
+      <formula1>'dataset_type'!$A$1:$A$55</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="F2:F1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'analyte_class'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="G2:G1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'is_targeted'!$A$1:$A$2</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="G2:G1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'acquisition_instrument_vendor'!$A$1:$A$30</formula1>
+    <dataValidation type="list" sqref="H2:H1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'acquisition_instrument_vendor'!$A$1:$A$33</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="H2:H1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'acquisition_instrument_model'!$A$1:$A$77</formula1>
+    <dataValidation type="list" sqref="I2:I1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'acquisition_instrument_model'!$A$1:$A$86</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="I2:I1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="J2:J1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
       <formula1>0</formula1>
       <formula2/>
     </dataValidation>
-    <dataValidation type="list" sqref="J2:J1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="K2:K1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'source_storage_duration_unit'!$A$1:$A$5</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="K2:K1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="L2:L1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
       <formula1>0</formula1>
       <formula2/>
     </dataValidation>
-    <dataValidation type="list" sqref="L2:L1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="M2:M1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'time_since_acquisition_instrume'!$A$1:$A$3</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="O2:O1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="P2:P1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'barcode_offset'!$A$1:$A$9</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="P2:P1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="Q2:Q1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'barcode_read'!$A$1:$A$3</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Q2:Q1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="R2:R1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'barcode_size'!$A$1:$A$6</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="R2:R1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="S2:S1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'umi_offset'!$A$1:$A$4</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="S2:S1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="T2:T1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'umi_read'!$A$1:$A$3</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="T2:T1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="U2:U1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'umi_size'!$A$1:$A$5</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="U2:U1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="V2:V1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'assay_input_entity'!$A$1:$A$5</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="between" sqref="V2:V1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
+    <dataValidation type="whole" operator="between" sqref="W2:W1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
       <formula1>-2147483648</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" sqref="W2:W1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
+    <dataValidation type="decimal" operator="between" sqref="X2:X1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
       <formula1>-3.4028235E38</formula1>
       <formula2>3.4028235E38</formula2>
     </dataValidation>
-    <dataValidation type="list" sqref="X2:X1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="Y2:Y1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'amount_of_input_analyte_unit'!$A$1:$A$2</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="between" sqref="Z2:Z1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
+    <dataValidation type="whole" operator="between" sqref="AA2:AA1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
       <formula1>-2147483648</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" sqref="AA2:AA1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
+    <dataValidation type="decimal" operator="between" sqref="AB2:AB1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
       <formula1>-3.4028235E38</formula1>
       <formula2>3.4028235E38</formula2>
     </dataValidation>
-    <dataValidation type="list" sqref="AB2:AB1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="AC2:AC1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'library_input_amount_unit'!$A$1:$A$2</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" sqref="AC2:AC1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
+    <dataValidation type="decimal" operator="between" sqref="AD2:AD1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
       <formula1>-3.4028235E38</formula1>
       <formula2>3.4028235E38</formula2>
     </dataValidation>
-    <dataValidation type="list" sqref="AD2:AD1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="AE2:AE1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'library_output_amount_unit'!$A$1:$A$2</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" sqref="AE2:AE1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
+    <dataValidation type="decimal" operator="between" sqref="AF2:AF1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
       <formula1>-3.4028235E38</formula1>
       <formula2>3.4028235E38</formula2>
     </dataValidation>
-    <dataValidation type="list" sqref="AF2:AF1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="AG2:AG1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'library_concentration_unit'!$A$1:$A$3</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="AG2:AG1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="AH2:AH1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'library_layout'!$A$1:$A$2</formula1>
-    </dataValidation>
-    <dataValidation type="whole" operator="between" sqref="AH2:AH1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
-      <formula1>-2147483648</formula1>
-      <formula2>2147483647</formula2>
     </dataValidation>
     <dataValidation type="whole" operator="between" sqref="AI2:AI1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
       <formula1>-2147483648</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" sqref="AJ2:AJ1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'library_preparation_kit'!$A$1:$A$37</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="AK2:AK1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'sample_indexing_kit'!$A$1:$A$19</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="AM2:AM1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'is_technical_replicate'!$A$1:$A$2</formula1>
-    </dataValidation>
-    <dataValidation type="whole" operator="between" sqref="AN2:AN1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
+    <dataValidation type="whole" operator="between" sqref="AJ2:AJ1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
       <formula1>-2147483648</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" sqref="AO2:AO1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="AK2:AK1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'library_preparation_kit'!$A$1:$A$38</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="AL2:AL1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'sample_indexing_kit'!$A$1:$A$19</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="AN2:AN1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'is_technical_replicate'!$A$1:$A$2</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="between" sqref="AO2:AO1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
+      <formula1>-2147483648</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="list" sqref="AP2:AP1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'sequencing_reagent_kit'!$A$1:$A$29</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="AS2:AS1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="AT2:AT1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'preparation_instrument_vendor'!$A$1:$A$11</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="AT2:AT1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="AU2:AU1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'preparation_instrument_model'!$A$1:$A$19</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="AU2:AU1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="AV2:AV1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'preparation_instrument_kit'!$A$1:$A$13</formula1>
     </dataValidation>
   </dataValidations>
@@ -2911,26 +3032,26 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>383</v>
+        <v>418</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>384</v>
+        <v>419</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>214</v>
+        <v>231</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>215</v>
+        <v>232</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>385</v>
+        <v>420</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>386</v>
+        <v>421</v>
       </c>
     </row>
   </sheetData>
@@ -2945,32 +3066,32 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>388</v>
+        <v>423</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>389</v>
+        <v>424</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>390</v>
+        <v>425</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>391</v>
+        <v>426</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>392</v>
+        <v>427</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>214</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -2985,22 +3106,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>374</v>
+        <v>409</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>389</v>
+        <v>424</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>394</v>
+        <v>429</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>214</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -3015,26 +3136,26 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>383</v>
+        <v>418</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>384</v>
+        <v>419</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>214</v>
+        <v>231</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>215</v>
+        <v>232</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>385</v>
+        <v>420</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>386</v>
+        <v>421</v>
       </c>
     </row>
   </sheetData>
@@ -3049,27 +3170,27 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>375</v>
+        <v>410</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>397</v>
+        <v>432</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>398</v>
+        <v>433</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>399</v>
+        <v>434</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>214</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -3084,42 +3205,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>401</v>
+        <v>436</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>402</v>
+        <v>437</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>403</v>
+        <v>438</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>404</v>
+        <v>439</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>405</v>
+        <v>440</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>406</v>
+        <v>441</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>407</v>
+        <v>442</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>408</v>
+        <v>443</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>409</v>
+        <v>444</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>410</v>
+        <v>445</v>
       </c>
     </row>
   </sheetData>
@@ -3134,18 +3255,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>414</v>
+        <v>449</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>415</v>
+        <v>450</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>416</v>
+        <v>451</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>417</v>
+        <v>452</v>
       </c>
     </row>
   </sheetData>
@@ -3160,18 +3281,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>422</v>
+        <v>457</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>423</v>
+        <v>458</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>416</v>
+        <v>451</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>417</v>
+        <v>452</v>
       </c>
     </row>
   </sheetData>
@@ -3186,18 +3307,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>422</v>
+        <v>457</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>423</v>
+        <v>458</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>416</v>
+        <v>451</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>417</v>
+        <v>452</v>
       </c>
     </row>
   </sheetData>
@@ -3212,26 +3333,26 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>428</v>
+        <v>463</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>429</v>
+        <v>464</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>430</v>
+        <v>465</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>431</v>
+        <v>466</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>432</v>
+        <v>467</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>433</v>
+        <v>468</v>
       </c>
     </row>
   </sheetData>
@@ -3241,415 +3362,447 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>105</v>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s" s="0">
+        <v>107</v>
+      </c>
+      <c r="B52" t="s" s="0">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s" s="0">
+        <v>109</v>
+      </c>
+      <c r="B53" t="s" s="0">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s" s="0">
+        <v>111</v>
+      </c>
+      <c r="B54" t="s" s="0">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="B55" t="s" s="0">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -3664,18 +3817,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>435</v>
+        <v>470</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>436</v>
+        <v>471</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>437</v>
+        <v>472</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>438</v>
+        <v>473</v>
       </c>
     </row>
   </sheetData>
@@ -3685,303 +3838,311 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>442</v>
+        <v>477</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>443</v>
+        <v>478</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>444</v>
+        <v>479</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>445</v>
+        <v>480</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>446</v>
+        <v>481</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>447</v>
+        <v>482</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>448</v>
+        <v>483</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>449</v>
+        <v>484</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>450</v>
+        <v>485</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>451</v>
+        <v>486</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>452</v>
+        <v>487</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>453</v>
+        <v>488</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>454</v>
+        <v>489</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>455</v>
+        <v>490</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>456</v>
+        <v>491</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>457</v>
+        <v>492</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>458</v>
+        <v>493</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>459</v>
+        <v>494</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>460</v>
+        <v>495</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>461</v>
+        <v>496</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>462</v>
+        <v>497</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>463</v>
+        <v>498</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>464</v>
+        <v>499</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>465</v>
+        <v>500</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>466</v>
+        <v>501</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>467</v>
+        <v>502</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>468</v>
+        <v>503</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>469</v>
+        <v>504</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>470</v>
+        <v>505</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>471</v>
+        <v>506</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>472</v>
+        <v>507</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>473</v>
+        <v>508</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>474</v>
+        <v>509</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>475</v>
+        <v>510</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>476</v>
+        <v>511</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>477</v>
+        <v>512</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>478</v>
+        <v>513</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>479</v>
+        <v>514</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>480</v>
+        <v>515</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>481</v>
+        <v>516</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>482</v>
+        <v>517</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>483</v>
+        <v>518</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>484</v>
+        <v>519</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>485</v>
+        <v>520</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>486</v>
+        <v>521</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>487</v>
+        <v>522</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>488</v>
+        <v>523</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>489</v>
+        <v>524</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>490</v>
+        <v>525</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>491</v>
+        <v>526</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>492</v>
+        <v>527</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>493</v>
+        <v>528</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>494</v>
+        <v>529</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>495</v>
+        <v>530</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>496</v>
+        <v>531</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>497</v>
+        <v>532</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>498</v>
+        <v>533</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>499</v>
+        <v>534</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>500</v>
+        <v>535</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>501</v>
+        <v>536</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>502</v>
+        <v>537</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>503</v>
+        <v>538</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>504</v>
+        <v>539</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>505</v>
+        <v>540</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>506</v>
+        <v>541</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>507</v>
+        <v>542</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>508</v>
+        <v>543</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>509</v>
+        <v>544</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>510</v>
+        <v>545</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>511</v>
+        <v>546</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>512</v>
+        <v>547</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>513</v>
+        <v>548</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>514</v>
+        <v>549</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>515</v>
+        <v>550</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="0">
+        <v>551</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>552</v>
       </c>
     </row>
   </sheetData>
@@ -3996,154 +4157,154 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>517</v>
+        <v>554</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>518</v>
+        <v>555</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>519</v>
+        <v>556</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>520</v>
+        <v>557</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>214</v>
+        <v>231</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>215</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>521</v>
+        <v>558</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>522</v>
+        <v>559</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>523</v>
+        <v>560</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>524</v>
+        <v>561</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>525</v>
+        <v>562</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>526</v>
+        <v>563</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>527</v>
+        <v>564</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>528</v>
+        <v>565</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>529</v>
+        <v>566</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>530</v>
+        <v>567</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>531</v>
+        <v>568</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>532</v>
+        <v>569</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>533</v>
+        <v>570</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>534</v>
+        <v>571</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>498</v>
+        <v>535</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>499</v>
+        <v>536</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>535</v>
+        <v>572</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>536</v>
+        <v>573</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>537</v>
+        <v>574</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>538</v>
+        <v>575</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>539</v>
+        <v>576</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>540</v>
+        <v>577</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>541</v>
+        <v>578</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>542</v>
+        <v>579</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>543</v>
+        <v>580</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>544</v>
+        <v>581</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>545</v>
+        <v>582</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>546</v>
+        <v>583</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>547</v>
+        <v>584</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>548</v>
+        <v>585</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>549</v>
+        <v>586</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>550</v>
+        <v>587</v>
       </c>
     </row>
   </sheetData>
@@ -4158,12 +4319,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>142</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>143</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -4178,234 +4339,234 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>555</v>
+        <v>592</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>556</v>
+        <v>593</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>557</v>
+        <v>594</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>558</v>
+        <v>595</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>559</v>
+        <v>596</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>560</v>
+        <v>597</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>561</v>
+        <v>598</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>562</v>
+        <v>599</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>563</v>
+        <v>600</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>564</v>
+        <v>601</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>565</v>
+        <v>602</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>566</v>
+        <v>603</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>567</v>
+        <v>604</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>568</v>
+        <v>605</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>569</v>
+        <v>606</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>570</v>
+        <v>607</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>571</v>
+        <v>608</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>572</v>
+        <v>609</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>573</v>
+        <v>610</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>574</v>
+        <v>611</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>575</v>
+        <v>612</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>576</v>
+        <v>613</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>577</v>
+        <v>614</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>578</v>
+        <v>615</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>579</v>
+        <v>616</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>580</v>
+        <v>617</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>581</v>
+        <v>618</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>582</v>
+        <v>619</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>583</v>
+        <v>620</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>584</v>
+        <v>621</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>585</v>
+        <v>622</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>586</v>
+        <v>623</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>587</v>
+        <v>624</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>588</v>
+        <v>625</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>498</v>
+        <v>535</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>499</v>
+        <v>536</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>589</v>
+        <v>626</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>590</v>
+        <v>627</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>591</v>
+        <v>628</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>592</v>
+        <v>629</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>593</v>
+        <v>630</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>594</v>
+        <v>631</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>595</v>
+        <v>632</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>596</v>
+        <v>633</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>597</v>
+        <v>634</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>598</v>
+        <v>635</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>599</v>
+        <v>636</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>600</v>
+        <v>637</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>601</v>
+        <v>638</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>602</v>
+        <v>639</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>603</v>
+        <v>640</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>604</v>
+        <v>641</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>605</v>
+        <v>642</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>606</v>
+        <v>643</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>607</v>
+        <v>644</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>608</v>
+        <v>645</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>609</v>
+        <v>646</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>610</v>
+        <v>647</v>
       </c>
     </row>
   </sheetData>
@@ -4420,90 +4581,90 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>176</v>
+        <v>189</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>194</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>214</v>
+        <v>231</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>215</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>150</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>615</v>
+        <v>652</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>616</v>
+        <v>653</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>617</v>
+        <v>654</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>618</v>
+        <v>655</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>198</v>
+        <v>215</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>202</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>174</v>
+        <v>185</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>162</v>
+        <v>173</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>619</v>
+        <v>656</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>620</v>
+        <v>657</v>
       </c>
     </row>
   </sheetData>
@@ -4518,154 +4679,154 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>286</v>
+        <v>311</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>287</v>
+        <v>312</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>214</v>
+        <v>231</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>215</v>
+        <v>232</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>622</v>
+        <v>659</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>623</v>
+        <v>660</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>218</v>
+        <v>235</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>219</v>
+        <v>236</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>624</v>
+        <v>661</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>625</v>
+        <v>662</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>498</v>
+        <v>535</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>499</v>
+        <v>536</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>266</v>
+        <v>291</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>267</v>
+        <v>292</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>343</v>
+        <v>378</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>344</v>
+        <v>379</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>626</v>
+        <v>663</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>627</v>
+        <v>664</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>628</v>
+        <v>665</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>629</v>
+        <v>666</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>630</v>
+        <v>667</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>631</v>
+        <v>668</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>632</v>
+        <v>669</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>633</v>
+        <v>670</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>634</v>
+        <v>671</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>635</v>
+        <v>672</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>636</v>
+        <v>673</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>637</v>
+        <v>674</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>638</v>
+        <v>675</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>639</v>
+        <v>676</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>640</v>
+        <v>677</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>641</v>
+        <v>678</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>642</v>
+        <v>679</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>643</v>
+        <v>680</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>644</v>
+        <v>681</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>645</v>
+        <v>682</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>646</v>
+        <v>683</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>647</v>
+        <v>684</v>
       </c>
     </row>
   </sheetData>
@@ -4680,106 +4841,106 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>649</v>
+        <v>686</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>650</v>
+        <v>687</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>651</v>
+        <v>688</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>652</v>
+        <v>689</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>494</v>
+        <v>531</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>495</v>
+        <v>532</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>653</v>
+        <v>690</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>654</v>
+        <v>691</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>655</v>
+        <v>692</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>656</v>
+        <v>693</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>657</v>
+        <v>694</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>658</v>
+        <v>695</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>498</v>
+        <v>535</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>499</v>
+        <v>536</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>659</v>
+        <v>696</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>660</v>
+        <v>697</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>661</v>
+        <v>698</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>662</v>
+        <v>699</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>508</v>
+        <v>545</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>509</v>
+        <v>546</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>663</v>
+        <v>700</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>664</v>
+        <v>701</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>665</v>
+        <v>702</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>666</v>
+        <v>703</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>667</v>
+        <v>704</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>668</v>
+        <v>705</v>
       </c>
     </row>
   </sheetData>
@@ -4800,30 +4961,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>671</v>
+        <v>708</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>672</v>
+        <v>709</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>674</v>
+        <v>711</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>676</v>
+        <v>713</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>673</v>
+        <v>710</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>675</v>
+        <v>712</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>677</v>
+        <v>714</v>
       </c>
     </row>
   </sheetData>
@@ -4833,143 +4994,151 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>108</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>110</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>112</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>116</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>118</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>120</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>122</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>124</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>126</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>128</v>
+        <v>137</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>130</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>132</v>
+        <v>141</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>134</v>
+        <v>143</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>136</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>138</v>
+        <v>147</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>140</v>
+        <v>149</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>150</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -4984,12 +5153,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>142</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>143</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -4999,247 +5168,271 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>146</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>148</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>150</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>152</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>154</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>156</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>158</v>
+        <v>169</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>160</v>
+        <v>171</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>162</v>
+        <v>173</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>164</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>166</v>
+        <v>177</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>168</v>
+        <v>179</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>170</v>
+        <v>181</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>172</v>
+        <v>183</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>174</v>
+        <v>185</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>176</v>
+        <v>187</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>178</v>
+        <v>189</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>180</v>
+        <v>191</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>182</v>
+        <v>193</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>184</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>186</v>
+        <v>197</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>188</v>
+        <v>199</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>190</v>
+        <v>201</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>192</v>
+        <v>203</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>194</v>
+        <v>205</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>196</v>
+        <v>207</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>198</v>
+        <v>209</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>200</v>
+        <v>211</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>201</v>
+        <v>212</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>202</v>
+        <v>213</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>204</v>
+        <v>215</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
+        <v>216</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -5249,623 +5442,695 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B77"/>
+  <dimension ref="A1:B86"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>206</v>
+        <v>223</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>207</v>
+        <v>224</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>208</v>
+        <v>225</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>209</v>
+        <v>226</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>210</v>
+        <v>227</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>211</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>212</v>
+        <v>229</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>213</v>
+        <v>230</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>214</v>
+        <v>231</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>215</v>
+        <v>232</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>216</v>
+        <v>233</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>217</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>218</v>
+        <v>235</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>219</v>
+        <v>236</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>220</v>
+        <v>237</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>221</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>222</v>
+        <v>239</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>223</v>
+        <v>240</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>224</v>
+        <v>241</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>225</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>226</v>
+        <v>243</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>227</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>228</v>
+        <v>245</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>229</v>
+        <v>246</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>230</v>
+        <v>247</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>231</v>
+        <v>248</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>232</v>
+        <v>249</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>233</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>234</v>
+        <v>251</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>235</v>
+        <v>252</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>236</v>
+        <v>253</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>237</v>
+        <v>254</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>238</v>
+        <v>255</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>239</v>
+        <v>256</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>240</v>
+        <v>257</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>241</v>
+        <v>258</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>242</v>
+        <v>259</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>243</v>
+        <v>260</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>244</v>
+        <v>261</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>245</v>
+        <v>262</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>246</v>
+        <v>263</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>247</v>
+        <v>264</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>248</v>
+        <v>265</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>249</v>
+        <v>266</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>250</v>
+        <v>267</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>251</v>
+        <v>268</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>252</v>
+        <v>269</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>253</v>
+        <v>270</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>254</v>
+        <v>271</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>255</v>
+        <v>272</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>256</v>
+        <v>273</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>257</v>
+        <v>274</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>258</v>
+        <v>275</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>259</v>
+        <v>276</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>260</v>
+        <v>277</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>261</v>
+        <v>278</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>262</v>
+        <v>279</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>263</v>
+        <v>280</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>264</v>
+        <v>281</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>265</v>
+        <v>282</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>266</v>
+        <v>283</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>267</v>
+        <v>284</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>268</v>
+        <v>285</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>269</v>
+        <v>286</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>270</v>
+        <v>287</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>271</v>
+        <v>288</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>272</v>
+        <v>289</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>273</v>
+        <v>290</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>274</v>
+        <v>291</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>275</v>
+        <v>292</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>276</v>
+        <v>293</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>277</v>
+        <v>294</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>278</v>
+        <v>295</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>279</v>
+        <v>296</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>280</v>
+        <v>297</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>281</v>
+        <v>298</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>282</v>
+        <v>299</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>283</v>
+        <v>300</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>284</v>
+        <v>301</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>285</v>
+        <v>302</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>286</v>
+        <v>303</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>287</v>
+        <v>304</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>288</v>
+        <v>305</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>289</v>
+        <v>306</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>290</v>
+        <v>307</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>291</v>
+        <v>308</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>292</v>
+        <v>309</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>293</v>
+        <v>310</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>294</v>
+        <v>311</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>295</v>
+        <v>312</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>296</v>
+        <v>313</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>297</v>
+        <v>314</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>298</v>
+        <v>315</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>299</v>
+        <v>316</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>300</v>
+        <v>317</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>301</v>
+        <v>318</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>302</v>
+        <v>319</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>303</v>
+        <v>320</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>304</v>
+        <v>321</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>305</v>
+        <v>322</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>306</v>
+        <v>323</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>307</v>
+        <v>324</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>308</v>
+        <v>325</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>309</v>
+        <v>326</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>310</v>
+        <v>327</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>311</v>
+        <v>328</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>312</v>
+        <v>329</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>313</v>
+        <v>330</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>314</v>
+        <v>331</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>315</v>
+        <v>332</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>316</v>
+        <v>333</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>317</v>
+        <v>334</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>318</v>
+        <v>335</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>319</v>
+        <v>336</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
-        <v>320</v>
+        <v>337</v>
       </c>
       <c r="B58" t="s" s="0">
-        <v>321</v>
+        <v>338</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
-        <v>322</v>
+        <v>339</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>323</v>
+        <v>340</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="0">
-        <v>70</v>
+        <v>341</v>
       </c>
       <c r="B60" t="s" s="0">
-        <v>324</v>
+        <v>342</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>325</v>
+        <v>343</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>326</v>
+        <v>344</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s" s="0">
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="B62" t="s" s="0">
-        <v>328</v>
+        <v>346</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="0">
-        <v>329</v>
+        <v>347</v>
       </c>
       <c r="B63" t="s" s="0">
-        <v>330</v>
+        <v>348</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s" s="0">
-        <v>175</v>
+        <v>349</v>
       </c>
       <c r="B64" t="s" s="0">
-        <v>176</v>
+        <v>350</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s" s="0">
-        <v>331</v>
+        <v>351</v>
       </c>
       <c r="B65" t="s" s="0">
-        <v>332</v>
+        <v>352</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s" s="0">
-        <v>333</v>
+        <v>353</v>
       </c>
       <c r="B66" t="s" s="0">
-        <v>334</v>
+        <v>354</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s" s="0">
-        <v>335</v>
+        <v>75</v>
       </c>
       <c r="B67" t="s" s="0">
-        <v>336</v>
+        <v>355</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s" s="0">
-        <v>337</v>
+        <v>356</v>
       </c>
       <c r="B68" t="s" s="0">
-        <v>338</v>
+        <v>357</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s" s="0">
-        <v>339</v>
+        <v>358</v>
       </c>
       <c r="B69" t="s" s="0">
-        <v>340</v>
+        <v>359</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s" s="0">
-        <v>341</v>
+        <v>360</v>
       </c>
       <c r="B70" t="s" s="0">
-        <v>342</v>
+        <v>361</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s" s="0">
-        <v>343</v>
+        <v>188</v>
       </c>
       <c r="B71" t="s" s="0">
-        <v>344</v>
+        <v>189</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s" s="0">
-        <v>345</v>
+        <v>362</v>
       </c>
       <c r="B72" t="s" s="0">
-        <v>346</v>
+        <v>363</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s" s="0">
-        <v>347</v>
+        <v>364</v>
       </c>
       <c r="B73" t="s" s="0">
-        <v>348</v>
+        <v>365</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s" s="0">
-        <v>349</v>
+        <v>366</v>
       </c>
       <c r="B74" t="s" s="0">
-        <v>350</v>
+        <v>367</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s" s="0">
-        <v>351</v>
+        <v>368</v>
       </c>
       <c r="B75" t="s" s="0">
-        <v>352</v>
+        <v>369</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s" s="0">
-        <v>353</v>
+        <v>370</v>
       </c>
       <c r="B76" t="s" s="0">
-        <v>354</v>
+        <v>371</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s" s="0">
-        <v>355</v>
+        <v>372</v>
       </c>
       <c r="B77" t="s" s="0">
-        <v>356</v>
+        <v>373</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s" s="0">
+        <v>374</v>
+      </c>
+      <c r="B78" t="s" s="0">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s" s="0">
+        <v>376</v>
+      </c>
+      <c r="B79" t="s" s="0">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s" s="0">
+        <v>378</v>
+      </c>
+      <c r="B80" t="s" s="0">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s" s="0">
+        <v>380</v>
+      </c>
+      <c r="B81" t="s" s="0">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="s" s="0">
+        <v>382</v>
+      </c>
+      <c r="B82" t="s" s="0">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="s" s="0">
+        <v>384</v>
+      </c>
+      <c r="B83" t="s" s="0">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s" s="0">
+        <v>386</v>
+      </c>
+      <c r="B84" t="s" s="0">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="s" s="0">
+        <v>388</v>
+      </c>
+      <c r="B85" t="s" s="0">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="s" s="0">
+        <v>390</v>
+      </c>
+      <c r="B86" t="s" s="0">
+        <v>391</v>
       </c>
     </row>
   </sheetData>
@@ -5880,42 +6145,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>359</v>
+        <v>394</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>360</v>
+        <v>395</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>361</v>
+        <v>396</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>362</v>
+        <v>397</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>363</v>
+        <v>398</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>364</v>
+        <v>399</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>365</v>
+        <v>400</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>366</v>
+        <v>401</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>367</v>
+        <v>402</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>368</v>
+        <v>403</v>
       </c>
     </row>
   </sheetData>
@@ -5930,26 +6195,26 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>361</v>
+        <v>396</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>362</v>
+        <v>397</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>363</v>
+        <v>398</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>364</v>
+        <v>399</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>365</v>
+        <v>400</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>366</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -5964,47 +6229,47 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>374</v>
+        <v>409</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>375</v>
+        <v>410</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>376</v>
+        <v>411</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>377</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>378</v>
+        <v>413</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>379</v>
+        <v>414</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>380</v>
+        <v>415</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>381</v>
+        <v>416</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>214</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>